<commit_message>
docs: dejar explícito que el catálogo es OpenMetrics v1, no PromQL v0
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/temporal-metrics-eval/metricas-temporal-cloud-openmetrics.xlsx
+++ b/temporal-metrics-eval/metricas-temporal-cloud-openmetrics.xlsx
@@ -765,7 +765,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>https://docs.temporal.io/cloud/metrics/openmetrics/metrics-reference  |  corte 2026-10-27</t>
+          <t>https://docs.temporal.io/cloud/metrics/openmetrics/metrics-reference  |  corte 2026-10-27. Esta es la referencia OpenMetrics vigente. NO usar https://docs.temporal.io/cloud/metrics/reference (catálogo PromQL v0).</t>
         </is>
       </c>
     </row>
@@ -777,19 +777,19 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>https://metrics.temporal.io/v1/metrics  (Bearer API key, rol Metrics Read-Only). Descriptores: https://metrics.temporal.io/v1/descriptors</t>
+          <t>https://metrics.temporal.io/v1/metrics  (Bearer API key, rol Metrics Read-Only). Descriptores: https://metrics.temporal.io/v1/descriptors. No es el endpoint PromQL /api/v1/query ni mTLS.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Convención v1</t>
+          <t>Generación</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Todas se exponen como gauge OpenMetrics. Rate = promedio /s en ventana de 1 min. Value = último agregado. Latency = percentil precalculado en segundos. NO usar rate().</t>
+          <t>Solo temporal_cloud_v1_*. OpenMetrics scrape. Rate = promedio /s en ventana de 1 min. Value = último agregado. Latency = percentil precalculado en segundos. NO usar rate().</t>
         </is>
       </c>
     </row>
@@ -820,12 +820,12 @@
     <row r="10" ht="36" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>PromQL v0</t>
+          <t>PromQL legado</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>temporal_cloud_v0_* apagado 5 oct 2026. No copiar alertas con rate() del mixin legado.</t>
+          <t>El endpoint PromQL (temporal_cloud_v0_*, mTLS) se deprecó el 2 abr 2026 y se apagó el 5 oct 2026. No hay series v0 en este Excel. La columna Query es PromQL de Grafana contra el scrape v1, no contra el endpoint muerto.</t>
         </is>
       </c>
     </row>
@@ -1506,7 +1506,7 @@
       </c>
       <c r="O1" s="5" t="inlineStr">
         <is>
-          <t>PromQL borrador (v1, sin rate())</t>
+          <t>Query Prometheus (scrape OpenMetrics v1, sin rate())</t>
         </is>
       </c>
       <c r="P1" s="5" t="inlineStr">
@@ -10718,7 +10718,7 @@
       </c>
       <c r="O1" s="5" t="inlineStr">
         <is>
-          <t>PromQL borrador (v1, sin rate())</t>
+          <t>Query Prometheus (scrape OpenMetrics v1, sin rate())</t>
         </is>
       </c>
       <c r="P1" s="5" t="inlineStr">
@@ -15233,7 +15233,7 @@
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>OpenMetrics metrics reference</t>
+          <t>OpenMetrics metrics reference (USAR)</t>
         </is>
       </c>
       <c r="B4" s="23" t="inlineStr">
@@ -15243,7 +15243,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Catálogo completo temporal_cloud_v1_* (este Excel).</t>
+          <t>Catálogo vigente temporal_cloud_v1_*. Única fuente de este Excel.</t>
         </is>
       </c>
     </row>
@@ -15260,7 +15260,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>API key, rol Metrics Read-Only, scrape.</t>
+          <t>API key, rol Metrics Read-Only, scrape a metrics.temporal.io.</t>
         </is>
       </c>
     </row>
@@ -15294,7 +15294,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Cuándo usar Cloud vs SDK.</t>
+          <t>Cuándo usar Cloud vs SDK. Apunta al catálogo OpenMetrics.</t>
         </is>
       </c>
     </row>
@@ -15328,73 +15328,90 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>No usar rate() en v1. PromQL v0 apagado 5 oct 2026.</t>
+          <t>PromQL endpoint deprecado 2 abr 2026, apagado 5 oct 2026. v0 counters → v1 rates. No rate().</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Endpoint métricas</t>
+          <t>NO USAR — metrics reference PromQL v0</t>
         </is>
       </c>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>https://metrics.temporal.io/v1/metrics</t>
+          <t>https://docs.temporal.io/cloud/metrics/reference</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Scrape Prometheus-compatible.</t>
+          <t>Catálogo legado temporal_cloud_v0_*. Endpoint PromQL + mTLS. Apagado 5 oct 2026.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Endpoint descriptores</t>
+          <t>Endpoint métricas</t>
         </is>
       </c>
       <c r="B11" s="23" t="inlineStr">
         <is>
-          <t>https://metrics.temporal.io/v1/descriptors</t>
+          <t>https://metrics.temporal.io/v1/metrics</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Catálogo programático (misma API key).</t>
+          <t>Scrape Prometheus-compatible.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Standalone Activities</t>
+          <t>Endpoint descriptores</t>
         </is>
       </c>
       <c r="B12" s="23" t="inlineStr">
         <is>
-          <t>https://docs.temporal.io/standalone-activity</t>
+          <t>https://metrics.temporal.io/v1/descriptors</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Placeholder __standalone_activity en labels.</t>
+          <t>Catálogo programático (misma API key).</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
+          <t>Standalone Activities</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>https://docs.temporal.io/standalone-activity</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Placeholder __standalone_activity en labels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
           <t>Alertas BCP (interno)</t>
         </is>
       </c>
-      <c r="B13" s="23" t="inlineStr">
+      <c r="B14" s="23" t="inlineStr">
         <is>
           <t>grafana-temporal/alertas-catalogo.yaml</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Reglas P1–P3 ya propuestas sobre este mismo set.</t>
         </is>
@@ -15422,6 +15439,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>